<commit_message>
correct error ref: duplicated rows
</commit_message>
<xml_diff>
--- a/ref/scTypeDB.xlsx
+++ b/ref/scTypeDB.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="602">
   <si>
     <t xml:space="preserve">tissueType</t>
   </si>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">PTPRC,GYPA,RUVBL1,TFRC,FOLR1,CD36,ITGA4,HBB,CD235a,HBD,CA1</t>
   </si>
   <si>
-    <t xml:space="preserve">Es</t>
+    <t xml:space="preserve">Eryth</t>
   </si>
   <si>
     <t xml:space="preserve">HSC/MPP cells</t>
@@ -2221,7 +2221,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E290"/>
+  <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="8.8515625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.85"/>
@@ -6344,14 +6344,16 @@
         <v>542</v>
       </c>
       <c r="B282" s="22" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C282" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="D282" s="25"/>
+        <v>90</v>
+      </c>
+      <c r="D282" s="22" t="s">
+        <v>91</v>
+      </c>
       <c r="E282" s="24" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6359,16 +6361,14 @@
         <v>542</v>
       </c>
       <c r="B283" s="22" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C283" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D283" s="22" t="s">
-        <v>91</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D283" s="25"/>
       <c r="E283" s="24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6376,14 +6376,14 @@
         <v>542</v>
       </c>
       <c r="B284" s="22" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="C284" s="22" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="D284" s="25"/>
       <c r="E284" s="24" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6391,14 +6391,14 @@
         <v>542</v>
       </c>
       <c r="B285" s="22" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C285" s="22" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D285" s="25"/>
       <c r="E285" s="24" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="286" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6406,14 +6406,14 @@
         <v>542</v>
       </c>
       <c r="B286" s="22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C286" s="22" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D286" s="25"/>
       <c r="E286" s="24" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6421,61 +6421,47 @@
         <v>542</v>
       </c>
       <c r="B287" s="22" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C287" s="22" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D287" s="25"/>
       <c r="E287" s="24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A288" s="21" t="s">
+      <c r="A288" s="26" t="s">
         <v>542</v>
       </c>
       <c r="B288" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C288" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D288" s="25"/>
       <c r="E288" s="24" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A289" s="26" t="s">
+      <c r="A289" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B289" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="C289" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="D289" s="25"/>
-      <c r="E289" s="24" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="290" customFormat="false" ht="13.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A290" s="2" t="s">
-        <v>542</v>
-      </c>
-      <c r="B290" s="26" t="s">
+      <c r="B289" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="C290" s="27" t="s">
+      <c r="C289" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="D290" s="28"/>
-      <c r="E290" s="29" t="s">
+      <c r="D289" s="28"/>
+      <c r="E289" s="29" t="s">
         <v>120</v>
       </c>
     </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.3"/>

</xml_diff>